<commit_message>
Ja casi ho tinc
--HG--
branch : Desgloç Per IRPF
</commit_message>
<xml_diff>
--- a/Docs/PiG-Hisenda.xlsx
+++ b/Docs/PiG-Hisenda.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF63FC0-2322-45C4-A876-759610FC7F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{427CD0B5-F052-461F-A30C-8B6D0989AF75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{862274CE-5946-45C0-85D2-512CA502EF5B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="24">
   <si>
     <t>Perdues Ant</t>
   </si>
@@ -104,6 +104,9 @@
   </si>
   <si>
     <t>APP</t>
+  </si>
+  <si>
+    <t>PiG+Div</t>
   </si>
 </sst>
 </file>
@@ -565,19 +568,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F7BAE93-4712-4139-A243-0172EF8EFE92}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.08984375" customWidth="1"/>
-    <col min="7" max="7" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.08984375" customWidth="1"/>
+    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -591,16 +595,19 @@
         <v>4</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2016</v>
       </c>
@@ -611,15 +618,19 @@
       <c r="D2" s="3">
         <v>54.08</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="G2" s="3">
+      <c r="E2" s="34">
+        <f>B2+D2</f>
+        <v>2809.21</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="H2" s="3">
         <v>2755.14</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="3">
         <v>52.5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2017</v>
       </c>
@@ -627,12 +638,16 @@
         <v>438.79</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="1"/>
-      <c r="G3" s="3">
+      <c r="E3" s="34">
+        <f t="shared" ref="E3:E7" si="0">B3+D3</f>
+        <v>438.79</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="H3" s="3">
         <v>438.81</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -643,17 +658,21 @@
       <c r="D4" s="3">
         <v>1.58</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="34">
+        <f t="shared" si="0"/>
+        <v>-1.5499999999999998</v>
+      </c>
+      <c r="F4" s="1">
         <v>0</v>
       </c>
-      <c r="G4" s="3">
+      <c r="H4" s="3">
         <v>-7.27</v>
       </c>
-      <c r="H4" s="3">
+      <c r="I4" s="3">
         <v>1.57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2019</v>
       </c>
@@ -663,17 +682,21 @@
       <c r="D5" s="3">
         <v>295.85000000000002</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="34">
+        <f t="shared" si="0"/>
+        <v>-8804.1299999999992</v>
+      </c>
+      <c r="F5" s="1">
         <v>0</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>-9095.86</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>294.32</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -684,15 +707,19 @@
         <v>3164</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="1">
+      <c r="E6" s="34">
+        <f t="shared" si="0"/>
+        <v>3164</v>
+      </c>
+      <c r="F6" s="1">
         <f>+B6-C6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>3125.41</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2021</v>
       </c>
@@ -705,30 +732,44 @@
       <c r="D7" s="4">
         <v>467.17</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="34">
+        <f t="shared" si="0"/>
+        <v>13408.86</v>
+      </c>
+      <c r="F7" s="1">
         <f>+B7-C7</f>
         <v>7095.9400000000005</v>
       </c>
-      <c r="G7" s="3">
+      <c r="H7" s="3">
         <v>12950.7</v>
       </c>
-      <c r="H7" s="3">
+      <c r="I7" s="3">
         <v>467.17</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C8" s="3"/>
       <c r="D8" s="4"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E8" s="4"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C7">

</xml_diff>